<commit_message>
Fix templates to exact column spec + add PDFs for easy opening
- Regenerate 3 templates with exact headers matching screenshots (Agile 8 cols, Defect 11 cols, UTP 6 cols) - ensures teacher requirement 100%
- Add exact-name files: Agile_Template_v0.1.xlsx, Defect_Tracker_Template_v0.1.xlsx, Unit_Test_Plan_v0.1.xlsx (plus _CoachAI_Completed aliases)
- Remove invalid .xlsm copy (was .xlsx data with .xlsm extension causing 'format and extension mismatch' error)
- Export PDFs (376KB, 294KB, 324KB) for users without Excel - opens anywhere
- Verified all xlsx open cleanly via Excel 16.0 COM (UsedRange rows 36/22/36)
- ASCII-safe content (no unicode arrows/Rs issues), Calibri, peach/blue headers, freeze panes, filters, print fit
</commit_message>
<xml_diff>
--- a/Doc/Agile_Template_v0.1_CoachAI_Completed.xlsx
+++ b/Doc/Agile_Template_v0.1_CoachAI_Completed.xlsx
@@ -88,18 +88,12 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -121,6 +115,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
         <bgColor rgb="00FFEB9C"/>
       </patternFill>
@@ -135,12 +135,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
         <bgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-        <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -186,17 +180,17 @@
   </cellStyleXfs>
   <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -205,8 +199,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -217,22 +217,16 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -602,7 +596,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -617,14 +611,14 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CoachAI — Product Backlog  (AI Customer Support Assistant with Live Response Guidance)</t>
+          <t>CoachAI - Product Backlog (AI Customer Support Assistant with Live Response Guidance)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Project: Development of AI-Powered Customer Support Assistant with Live Response Guidance  |  Team: CoachAI (Jun–Aug 2026 Batch)  |  Repo: github.com/MasterJi27  |  Deadline: 28-Aug-2026  |  Total Sprints: 6  |  Duration: 6 weeks</t>
+          <t>Project: Development of AI-Powered Customer Support Assistant with Live Response Guidance | Batch: Jun-Aug 2026 | Team: MasterJi27 + CoachAI Team | Repo: github.com/MasterJi27 | Sprints: 6 (6 weeks) | Deadline: 28-Aug-2026</t>
         </is>
       </c>
     </row>
@@ -687,7 +681,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>As a stakeholder, I want project charter &amp; requirement analysis so that scope, problem (late coaching, scattered KB, late escalation) and solution (real-time copilot) are documented</t>
+          <t>As a stakeholder, I want project charter and requirement analysis covering problem (late coaching, scattered KB, late escalation) and solution (real-time copilot) so scope is clear</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -712,20 +706,20 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>US-002</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>As a developer, I want GitHub repo with branching, .gitignore, MIT license &amp; README so that collaboration and versioning are enabled</t>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>As a developer, I want GitHub repo with branching, .gitignore, MIT license and README skeleton so collaboration is enabled</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -733,12 +727,12 @@
           <t>MUST HAVE</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>US-001</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>Team Lead</t>
         </is>
@@ -749,7 +743,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6" t="n">
         <v>1</v>
       </c>
@@ -763,7 +757,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>As an architect, I want system architecture design (React+Node+Python+Postgres+LLM chain Azure→OpenRouter→Groq) &amp; per-turn flow documented</t>
+          <t>As an architect, I want system architecture (React + Node + Python + Postgres + LLM chain Azure -&gt; OpenRouter -&gt; Groq) and 9-step per-turn flow documented</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -787,21 +781,21 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="6" t="n">
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>US-004</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>As a DevOps, I want environment config (.env.example, DATABASE_URL, AZURE/GROQ/OPENROUTER keys, COMPOSIO keys) with graceful degradation if keys missing</t>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>As DevOps, I want env config (.env.example, DATABASE_URL, AZURE/GROQ/OPENROUTER keys, COMPOSIO keys) with graceful degradation if keys missing</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -809,12 +803,12 @@
           <t>MUST HAVE</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>US-002</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>Backend Team</t>
         </is>
@@ -839,7 +833,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>As a PM, I want Orchestrator &amp; ConversationManager session lifecycle designed (start/process/advance/end + rehydration) for serverless</t>
+          <t>As PM, I want Orchestrator and ConversationManager session lifecycle (start/process/advance/end + rehydration via full_state JSON) for serverless</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -864,20 +858,20 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>US-006</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>As an agent, I want Customer Simulator (LLM temp 0.8, Hinglish ≤140 chars, sentiment state machine, 6 fallback scenarios) so training is realistic</t>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>As agent, I want Customer Simulator (LLM temp 0.8, Hinglish &lt;=140 chars, sentiment state machine, 6 fallbacks) for realistic training</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -885,12 +879,12 @@
           <t>MUST HAVE</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>US-005</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
@@ -915,7 +909,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>As an agent, I want Intent &amp; Sentiment Agent (intent + frustration 0-1 + satisfaction trend -1..1, JSON parsing with regex fallback) in &lt;0.5s</t>
+          <t>As agent, I want Intent and Sentiment Agent (intent + frustration 0-1 + trend -1..1, JSON regex fallback) in &lt;0.5s</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -939,21 +933,21 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="6" t="n">
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>US-008</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>As a manager, I want Escalation Monitor (weighted rule: frustration×0.4 + sentiment×0.2 + trend×0.15 + keywords×0.1 + length×0.1 + repetition×0.05) to flag risk</t>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>As manager, I want Escalation Monitor (weighted: frustration*0.4 + sentiment*0.2 + trend*0.15 + keywords*0.1 + length*0.1 + repetition*0.05)</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -961,12 +955,12 @@
           <t>MUST HAVE</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>US-007</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="10" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
@@ -991,7 +985,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>As an agent, I want Coaching Suggestion Agent (suggested reply + tone/clarity 1-5 + macros library + retention-code nudges) to guide reply before send</t>
+          <t>As agent, I want Coaching Suggestion (suggested reply + tone/clarity 1-5 + macros library + retention STAY15) before send</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -1015,21 +1009,21 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="6" t="n">
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B14" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>US-010</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>As a QA, I want Post-Interaction Summary Agent (overall = resolution×0.5 + coaching×0.3 + clarity/CSAT×0.2) &amp; PerformanceReport with gaps &amp; coaching tips</t>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>As QA, I want Post-Interaction Summary (overall = resolution*0.5 + coaching*0.3 + clarity*0.2) and PerformanceReport</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -1037,12 +1031,12 @@
           <t>MUST HAVE</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>US-009</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="10" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
@@ -1067,7 +1061,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>As a KB admin, I want RAG ingestion (.txt/.pdf via PyPDF2/.docx/.json/.md/.csv/.html) with paragraph→512-char chunking &amp; sentence re-split</t>
+          <t>As KB admin, I want RAG ingestion (.txt/.pdf/.docx/.json/.md/.csv/.html) with paragraph -&gt; 512-char chunks and sentence re-split</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -1091,21 +1085,21 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="6" t="n">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B16" s="6" t="n">
+      <c r="B16" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>US-012</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>As an agent, I want hybrid retrieval: semantic (OpenRouter nvidia/nemotron-3-embed-1b 2048d cosine, lazy embed, JSONB cache) + BM25/keyword offline fallback</t>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>As agent, I want hybrid retrieval: semantic (OpenRouter nemotron 2048d cosine, JSONB cache) + BM25/keyword offline fallback</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -1113,12 +1107,12 @@
           <t>MUST HAVE</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>US-011</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="10" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
@@ -1129,7 +1123,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="22" customHeight="1">
       <c r="A17" s="6" t="n">
         <v>3</v>
       </c>
@@ -1143,7 +1137,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>As an agent, I want Knowledge Recommendation Agent (agentic RAG synthesis → 1 distilled tip) + KB-gap detection (&lt;0.45 → pending FAQ draft via Auto-KB)</t>
+          <t>As agent, I want Knowledge Recommendation (agentic RAG 1 tip) + KB-gap &lt;0.45 -&gt; pending FAQ draft via Auto-KB</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -1167,34 +1161,34 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="6" t="n">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="6" t="n">
+      <c r="B18" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>US-014</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>As a manager, I want Deep Analysis Agent (1 LLM call → predicted CSAT 1-5, churn %, viral/PR risk + PR statement, fraud+protocol, defection+counter-offer, mind-read monologue)</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>As manager, I want Deep Analysis (1 LLM call -&gt; CSAT 1-5, churn %, viral/PR + statement, fraud+protocol, defection+offer, mind-read)</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>SHOULD HAVE</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>US-007</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
@@ -1205,7 +1199,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="22" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>3</v>
       </c>
@@ -1219,10 +1213,10 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>As a risk analyst, I want Predictive CSAT, Competitor Defection (keyword swiggy/zepto pre-scan), Viral Threat, Fraud Detector agents (each with LLM + keyword pre-scan)</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
+          <t>As analyst, I want Predictive CSAT, Defection (swiggy/zepto keywords), Viral Threat, Fraud Detector agents</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>SHOULD HAVE</t>
         </is>
@@ -1244,33 +1238,33 @@
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="6" t="n">
+      <c r="A20" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B20" s="6" t="n">
+      <c r="B20" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>US-016</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>As an agent, I want Customer Mind Reader (unstated intent), Multiverse Simulator (2-3 what-if replies with predicted CSAT), Cognitive Load, Patience Clock, Bot Agent (scripted Zomato menu, escalate on 'human' or frustration ≥0.7)</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>As agent, I want Mind Reader, Multiverse (2-3 what-if branches + CSAT), Cognitive Load, Patience Clock, Bot Agent (Zomato menu, escalate on human/frustration&gt;=0.7)</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>SHOULD HAVE</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>US-014</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G20" s="10" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
@@ -1295,10 +1289,10 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>As an agent, I want Manager Supervisor (whisper/takeover if frustration/escalation ≥0.5), Compliance Monitor (KB policy check), Tone Rewriter (&lt;10 chars → canned apology), Auto-Pilot (one-click reply + refund/voucher action)</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
+          <t>As agent, I want Manager Supervisor (whisper/takeover if &gt;=0.5), Compliance Monitor, Tone Rewriter (&lt;10 chars -&gt; canned apology), Auto-Pilot (one-click refund/voucher)</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>SHOULD HAVE</t>
         </is>
@@ -1319,34 +1313,34 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="6" t="n">
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B22" s="6" t="n">
+      <c r="B22" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>US-018</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>As a manager, I want Jira Bug Generator (transcript→structured ticket), Scenario Generator (LLM training scenarios), QA Audit Agent (21 ISO checks, pass if overall ≥0.75)</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>As manager, I want Jira Generator (transcript -&gt; ticket), Scenario Generator, QA Audit (21 checks, pass if overall&gt;=0.75)</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>SHOULD HAVE</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>US-010</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="10" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
@@ -1357,7 +1351,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="28" customHeight="1">
+    <row r="23" ht="22" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>4</v>
       </c>
@@ -1371,10 +1365,10 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>As an integrator, I want Composio backend (JIRA_CREATE_ISSUE, GMAIL_CREATE_EMAIL_DRAFT, Slack post) + mock_backend (lookup_order, process_refund &gt;₹500 supervisor guard, grant_voucher) with graceful fail</t>
-        </is>
-      </c>
-      <c r="E23" s="10" t="inlineStr">
+          <t>As integrator, I want Composio (JIRA_CREATE_ISSUE, GMAIL, Slack) + mock_backend (refund Rs.500 guard, voucher) with graceful fail</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>COULD HAVE</t>
         </is>
@@ -1395,34 +1389,34 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="6" t="n">
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B24" s="6" t="n">
+      <c r="B24" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>US-020</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>As a trainee, I want Survival Mode arcade (4 tickets, keyword-graded 0.85/0.6/0.35, HP/score/streak/power-ups, +500 bonus) &amp; Hall of Fame/Shame archive (≥0.85 / ≤0.45)</t>
-        </is>
-      </c>
-      <c r="E24" s="10" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>As trainee, I want Survival Mode (4 tickets, grading 0.85/0.6/0.35, HP/streak/power-ups +500) and Hall of Fame/Shame (&gt;=0.85 / &lt;=0.45)</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
         <is>
           <t>COULD HAVE</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>US-010</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G24" s="10" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
@@ -1433,7 +1427,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="22" customHeight="1">
       <c r="A25" s="6" t="n">
         <v>5</v>
       </c>
@@ -1447,7 +1441,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>As a frontend user, I want Node Express backend (auth register/login/guest/me/logout, sessionStore rehydration via pg JSONB, coaching.js, reports, scenarios, integrations) on port 8000</t>
+          <t>As user, I want Node Express backend (auth register/login/guest/me, sessionStore pg rehydration, 40+ routes, rag BM25, llm chain) port 8000</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -1471,21 +1465,21 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="6" t="n">
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B26" s="6" t="n">
+      <c r="B26" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>US-022</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>As a developer, I want Python FastAPI backend (server.py + features.py ~20 routes, _serialize_turn, /api/chat/*, /api/analysis/*) &amp; Streamlit app (src/ui/app.py 5 pages)</t>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>As dev, I want Python FastAPI (server.py + features.py 20 routes, _serialize_turn) and Streamlit app (src/ui/app.py 5 pages)</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -1493,12 +1487,12 @@
           <t>MUST HAVE</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>US-021</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G26" s="10" t="inlineStr">
         <is>
           <t>Backend Team</t>
         </is>
@@ -1523,7 +1517,7 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>As an agent, I want React frontend (Vite 5, Tailwind, react-router 6, framer-motion, @tanstack/react-query) with Landing/Login/Dashboard Coaching Console (Signals→KB→Reply→Risk)/Setup/Reports/Analytics/Knowledge/HallOfFame/JiraBoard</t>
+          <t>As agent, I want React frontend (Vite 5 + Tailwind + react-router 6, framer-motion, query) with Landing/Login/Dashboard (Signals/KB/Reply/Risk)/Setup/Reports/Analytics/Knowledge/HallOfFame/Jira</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -1547,21 +1541,21 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="6" t="n">
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B28" s="6" t="n">
+      <c r="B28" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>US-024</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>As a user, I want API integration (single fetch wrapper lib/api.js + bearer token), session/start, chat/message→coachTurn, chat/autopilot, manager-takeover, chat/end→email report</t>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>As user, I want API integration (api.js bearer), session/start, chat/message -&gt; coachTurn, autopilot, manager-takeover, chat/end -&gt; email report</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -1569,12 +1563,12 @@
           <t>MUST HAVE</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>US-023</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G28" s="10" t="inlineStr">
         <is>
           <t>Frontend Team</t>
         </is>
@@ -1585,7 +1579,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="22" customHeight="1">
       <c r="A29" s="6" t="n">
         <v>5</v>
       </c>
@@ -1599,10 +1593,10 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>As a power user, I want Feature Lab (Multiverse, Tone Rewriter, Compliance, Jira generator, TTS fish-audio→gTTS fallback, Survival Game) &amp; cross-session analytics &amp; jsPDF export</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="inlineStr">
+          <t>As power user, I want Feature Lab (Multiverse/Tone/Compliance/Jira), TTS fallback, Survival, analytics and jsPDF export</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>SHOULD HAVE</t>
         </is>
@@ -1624,20 +1618,20 @@
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="6" t="n">
+      <c r="A30" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B30" s="6" t="n">
+      <c r="B30" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>US-026</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>As a QA, I want test suites: pytest (14 tests + load, agents/RAG), vitest 7 tests, node --test, with CI on git push</t>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>As QA, I want tests: pytest 14 + load, vitest 7, node --test, CI on push</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -1645,12 +1639,12 @@
           <t>MUST HAVE</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>US-022</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G30" s="10" t="inlineStr">
         <is>
           <t>QA Team</t>
         </is>
@@ -1661,7 +1655,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="28" customHeight="1">
+    <row r="31" ht="22" customHeight="1">
       <c r="A31" s="6" t="n">
         <v>6</v>
       </c>
@@ -1675,7 +1669,7 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>As a DevOps, I want deployment: Vercel (frontend + Node backend), Streamlit Cloud, Neon/Supabase Postgres, plus health check /health (engine/RAG/db status)</t>
+          <t>As DevOps, I want deploy: Vercel (frontend+backend), Streamlit Cloud, Neon Postgres, /health (engine/RAG/db)</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -1699,21 +1693,21 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="6" t="n">
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B32" s="6" t="n">
+      <c r="B32" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>US-028</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>As a stakeholder, I want documentation deliverables: 10-slide PPT, KT Guide + Q&amp;A Bank (25 Qs), HTML browser docs, Deep Dive, Meeting CheatSheet, File Structure PDFs</t>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>As stakeholder, I want docs: 10-slide PPT exactly, KT Guide + Q&amp;A Bank 25 Qs, HTML docs, Deep Dive, CheatSheet</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -1721,12 +1715,12 @@
           <t>MUST HAVE</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F32" s="9" t="inlineStr">
         <is>
           <t>No Dependency</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G32" s="10" t="inlineStr">
         <is>
           <t>Team Lead</t>
         </is>
@@ -1737,7 +1731,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="28" customHeight="1">
+    <row r="33" ht="22" customHeight="1">
       <c r="A33" s="6" t="n">
         <v>6</v>
       </c>
@@ -1751,7 +1745,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>As a QA, I want hardening: ephemeral filesystem fix (DB authoritative), two-backends-one-Vercel-project guard, every LLM agent heuristic fallback, load testing</t>
+          <t>As QA, I want hardening: ephemeral FS fix (DB authoritative), two-backends-one-Vercel guard, all agents fallback, load test</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -1775,21 +1769,21 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="6" t="n">
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B34" s="6" t="n">
+      <c r="B34" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>US-030</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>As a PM, I want final packaging: Agile/Defect/UTP templates completed, GitHub release final/main, demo script (5 min Guest→Setup→Autopilot→FeatureLab→Reports), submission 28-Aug-2026</t>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>As PM, I want final packaging: templates filled, GitHub release final/main, 5-min demo script, submit 28-Aug-2026</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -1797,12 +1791,12 @@
           <t>MUST HAVE</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>US-028</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G34" s="10" t="inlineStr">
         <is>
           <t>Team Lead</t>
         </is>
@@ -1814,9 +1808,9 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
-        <is>
-          <t>Note: 30 user stories across 6 sprints (Agile Template v0.1). MoSCoW priority applied. All stories marked 3-Completed for final submission (28-Aug-2026). For reference, Sample_Agile.xls &amp; Agile_Template.xlsm are NOT to be uploaded/edited — this file is the submission-ready completed version for CoachAI (github.com/MasterJi27).</t>
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Note: 30 user stories across 6 sprints (Agile Template v0.1). MoSCoW applied. All 3-Completed for 28-Aug-2026 submission. Reference files Sample_Agile.xls and Agile_Template.xlsm NOT uploaded/edited - this file is the completed submission for CoachAI (github.com/MasterJi27).</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1822,6 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1841,7 +1834,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
@@ -1857,14 +1850,14 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CoachAI — Sprint Backlog (Task Breakdown, 6 Sprints — Jun-Aug 2026 Batch)</t>
+          <t>CoachAI - Sprint Backlog (Task Breakdown, 6 Sprints)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sprint-wise task decomposition with effort estimate (hrs), owner &amp; acceptance criteria — maps Product Backlog US-IDs to executable tasks</t>
+          <t>Sprint-wise tasks with effort (hrs), owner and acceptance criteria -&gt; maps US-IDs to executable tasks</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1927,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Requirement workshop, Infosys problem statement analysis, define MVP scope &amp; acceptance criteria</t>
+          <t>Requirement workshop, Infosys problem analysis, MVP scope and acceptance criteria</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -1950,7 +1943,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
@@ -1960,36 +1953,36 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>T-02</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>US-002</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Init GitHub repo, setup .gitignore, branch main, add MIT license, draft README structure</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Init GitHub repo, .gitignore, branch main, MIT license, README structure</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Team Lead</t>
         </is>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H6" s="12" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>T-01</t>
         </is>
@@ -2016,7 +2009,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Draw architecture diagram (React↔Node↔Python↔Postgres↔LLM), per-turn flow 9 steps, document in KT guide</t>
+          <t>Draw architecture (React-Node-Python-Postgres-LLM) and 9-step flow, document in KT guide</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -2042,36 +2035,36 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>T-04</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>US-004</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>Create .env.example (all 15 keys), implement config.py with 3-layer fallback (settings→env→st.secrets)</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Create .env.example (15 keys), config.py with 3-layer fallback (settings-&gt;env-&gt;st.secrets)</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>Backend Team</t>
         </is>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>T-02</t>
         </is>
@@ -2098,7 +2091,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Code Orchestrator (singleton, start_session, process_customer_input, rehydrate via full_state JSON) + ConversationManager</t>
+          <t>Code Orchestrator singleton + ConversationManager (rehydrate via full_state JSON)</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -2124,36 +2117,36 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>T-06</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>US-006</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Build customer_simulator agent: 6 fallback scenarios, Hinglish mixer, sentiment state machine, ≤140 chars guard</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Build customer_simulator: 6 fallbacks, Hinglish mixer, sentiment machine, &lt;=140 chars</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="H10" s="12" t="inlineStr">
+      <c r="H10" s="9" t="inlineStr">
         <is>
           <t>T-05</t>
         </is>
@@ -2180,7 +2173,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Build intent_sentiment agent: system prompt builder, LLM call temp 0.1, JSON parse regex, frustration/trend heuristics</t>
+          <t>Build intent_sentiment: builder, temp 0.1, JSON regex, frustration/trend heuristics</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -2206,36 +2199,36 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="12" t="n">
+      <c r="A12" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>T-08</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>US-008</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Build escalation_monitor: weighted formula implementation + unit tests (6 scenarios)</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Build escalation_monitor weighted formula + 6 unit tests</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>T-07</t>
         </is>
@@ -2262,7 +2255,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Build coaching_suggestion: macros library inject, tone/clarity heuristics + LLM synthesis, retention STAY15 logic</t>
+          <t>Build coaching_suggestion: macros inject, tone/clarity + LLM, STAY15 logic</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -2288,36 +2281,36 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="12" t="n">
+      <c r="A14" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>T-10</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>US-010</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>Build post_interaction_summary: overall_score formula, sentiment journey, auto-KB trigger on resolved+gap</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Build post_interaction_summary scoring + report JSON</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="G14" s="12" t="n">
+      <c r="G14" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>T-09</t>
         </is>
@@ -2344,7 +2337,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Implement rag/ingest.py: support 7 formats, paragraph→512 chunk, sentence re-split, ingest_directory</t>
+          <t>Implement ingest.py: 7 formats, para-&gt;512 chunks, sentence re-split</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -2370,36 +2363,36 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="12" t="n">
+      <c r="A16" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>T-12</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>US-012</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
-        <is>
-          <t>Implement hybrid search: embed_text (OpenRouter), cosine, BM25/keyword fallback, JSONB cache in Postgres</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Implement hybrid search: embed cosine, BM25 fallback, JSONB cache</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="F16" s="12" t="n">
+      <c r="F16" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="G16" s="12" t="n">
+      <c r="G16" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>T-11</t>
         </is>
@@ -2426,7 +2419,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Build knowledge_recommendation + KB-gap &lt;0.45 + auto_kb_agent drafting pending FAQ JSON</t>
+          <t>Build knowledge_recommendation + gap &lt;0.45 + auto_kb draft</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -2452,36 +2445,36 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="12" t="n">
+      <c r="A18" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>T-14</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>US-014</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Build deep_analysis: single LLM call prompt merging CSAT/churn/viral/PR/fraud/defection/mind-read, dict return + tests</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Build deep_analysis 1-call (CSAT/churn/viral/PR/fraud/defection/mind-read)</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F18" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="G18" s="12" t="n">
+      <c r="G18" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="H18" s="12" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>T-07</t>
         </is>
@@ -2508,7 +2501,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Build predictive_csat, competitor_defection, viral_threat, fraud_detector (keyword pre-scan → LLM with seeded defaults)</t>
+          <t>Build predictive_csat, defection, viral, fraud (keyword pre-scan -&gt; LLM)</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -2534,36 +2527,36 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="12" t="n">
+      <c r="A20" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>T-16</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>US-016</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
-        <is>
-          <t>Build mind_reader, multiverse_simulator (3 branches empathetic/rigid), cognitive_load, patience_clock, bot_agent (menu + escalate rules)</t>
-        </is>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Build mind_reader, multiverse (3 branches), cognitive, patience, bot menu</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="F20" s="12" t="n">
+      <c r="F20" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="G20" s="12" t="n">
+      <c r="G20" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="H20" s="12" t="inlineStr">
+      <c r="H20" s="9" t="inlineStr">
         <is>
           <t>T-14</t>
         </is>
@@ -2590,7 +2583,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Build manager_supervisor (≥0.5 no-op fast-path), compliance_monitor, tone_rewriter (&lt;10 chars guard), auto_pilot (mock + Composio email/Slack)</t>
+          <t>Build manager_supervisor (&gt;=0.5 no-op), compliance, tone_rewriter (&lt;10 guard), auto_pilot</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -2616,36 +2609,36 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="12" t="n">
+      <c r="A22" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>T-18</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>US-018</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>Build jira_bug_generator, scenario_generator, qa_audit (21 checks, pass ≥0.75), wire Composio + mock tools</t>
-        </is>
-      </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>Build jira_bug_generator, scenario_generator, qa_audit (21 checks, pass &gt;=0.75)</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="F22" s="12" t="n">
+      <c r="F22" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="G22" s="12" t="n">
+      <c r="G22" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="H22" s="12" t="inlineStr">
+      <c r="H22" s="9" t="inlineStr">
         <is>
           <t>T-10</t>
         </is>
@@ -2672,7 +2665,7 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Implement tools layer: mock_backend (₹500 guard) + composio_backend graceful degradation, feature flags</t>
+          <t>Implement mock_backend (Rs.500 guard) + composio_backend graceful fail</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -2698,36 +2691,36 @@
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="12" t="n">
+      <c r="A24" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>T-20</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>US-020</t>
         </is>
       </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>Build survival_game (4 tickets, grading 0.85/0.6/0.35, shield@3 streak, bonus+500) + hall_of_fame archiver</t>
-        </is>
-      </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>Build survival_game (4 tickets, 0.85/0.6/0.35, shield@3, +500) + hall_of_fame</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="F24" s="12" t="n">
+      <c r="F24" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="G24" s="12" t="n">
+      <c r="G24" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="H24" s="12" t="inlineStr">
+      <c r="H24" s="9" t="inlineStr">
         <is>
           <t>T-10</t>
         </is>
@@ -2754,7 +2747,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Build Node Express backend: auth (JWT-ish), sessionStore pg rehydration, 40+ routes in app.js, rag.js BM25, llm.js chain</t>
+          <t>Build Node Express backend: auth, sessionStore pg rehydration, 40+ routes</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -2780,36 +2773,36 @@
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="12" t="n">
+      <c r="A26" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>T-22</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>US-022</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
-        <is>
-          <t>Build Python FastAPI server.py + features.py (20 analysis routes), _serialize_turn, survival singleton, Streamlit app wiring</t>
-        </is>
-      </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>Build Python FastAPI (server+features 20 routes, _serialize_turn) + Streamlit</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>Backend Team</t>
         </is>
       </c>
-      <c r="F26" s="12" t="n">
+      <c r="F26" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="G26" s="12" t="n">
+      <c r="G26" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="H26" s="12" t="inlineStr">
+      <c r="H26" s="9" t="inlineStr">
         <is>
           <t>T-21</t>
         </is>
@@ -2836,7 +2829,7 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Build React frontend (Vite+Tailwind, 10 pages, code-split 58%), design system dark navy glassmorphism, api.js bearer wrapper</t>
+          <t>Build React frontend (Vite+Tailwind, 10 pages, 58% code-split) dark navy glassmorphism</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -2862,36 +2855,36 @@
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="12" t="n">
+      <c r="A28" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>T-24</t>
         </is>
       </c>
-      <c r="C28" s="12" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>US-024</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>Integrate frontend↔backend: Login/guest, Setup→Dashboard live 4-tab rail, Autopilot, Manager takeover, chat/end email</t>
-        </is>
-      </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Integrate frontend-backend: Login/guest, Setup-&gt;Dashboard 4-tab, Autopilot, takeover, end email</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t>Frontend Team</t>
         </is>
       </c>
-      <c r="F28" s="12" t="n">
+      <c r="F28" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="G28" s="12" t="n">
+      <c r="G28" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="H28" s="12" t="inlineStr">
+      <c r="H28" s="9" t="inlineStr">
         <is>
           <t>T-23</t>
         </is>
@@ -2918,7 +2911,7 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Build Feature Lab, Analytics, Reports jsPDF export, Knowledge admin (search debugger / chunk simulator / index doc)</t>
+          <t>Build Feature Lab, Analytics, Reports jsPDF, Knowledge admin tabs</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -2944,36 +2937,36 @@
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="12" t="n">
+      <c r="A30" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>T-26</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>US-026</t>
         </is>
       </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>Write &amp; run tests: pytest 14 + load, vitest 7 (Toast/ErrorBoundary/Jira), node --test, fix flaky LLM mocks</t>
-        </is>
-      </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>Write tests: pytest 14 + load, vitest 7, node --test</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>QA Team</t>
         </is>
       </c>
-      <c r="F30" s="12" t="n">
+      <c r="F30" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="G30" s="12" t="n">
+      <c r="G30" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="H30" s="12" t="inlineStr">
+      <c r="H30" s="9" t="inlineStr">
         <is>
           <t>T-22</t>
         </is>
@@ -3000,7 +2993,7 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Deploy to Vercel (frontend + backend), Streamlit Cloud, Neon Postgres; verify /health, fix ephemeral FS (DB authoritative)</t>
+          <t>Deploy: Vercel (frontend+backend), Streamlit Cloud, Neon Postgres, /health</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
@@ -3026,38 +3019,38 @@
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="12" t="n">
+      <c r="A32" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>T-28</t>
         </is>
       </c>
-      <c r="C32" s="12" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>US-028</t>
         </is>
       </c>
-      <c r="D32" s="13" t="inlineStr">
-        <is>
-          <t>Create deliverables: PPT 10 slides, KT Guide 342 lines, HTML docs, Deep Dive 429 lines, CheatSheet, QA Bank 25 Qs</t>
-        </is>
-      </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Create docs: PPT 10 slides exactly, KT Guide 342 lines, HTML docs, Deep Dive, QA Bank 25 Qs</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>Team Lead</t>
         </is>
       </c>
-      <c r="F32" s="12" t="n">
+      <c r="F32" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="G32" s="12" t="n">
+      <c r="G32" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="H32" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr">
@@ -3082,7 +3075,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Hardening: Vercel two-backends guard, all agents fallback verification, load test, .gitignore fix for Doc PDFs</t>
+          <t>Hardening: two-backends guard, ephemeral FS -&gt; DB, all fallbacks, load test</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
@@ -3108,36 +3101,36 @@
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="12" t="n">
+      <c r="A34" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>T-30</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>US-030</t>
         </is>
       </c>
-      <c r="D34" s="13" t="inlineStr">
-        <is>
-          <t>Package submission: fill Agile/Defect/UTP templates, GitHub push final/main, rehearse 10min demo flow, submit 28-Aug</t>
-        </is>
-      </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>Package: fill Agile/Defect/UTP, GitHub push final/main, rehearse 10min demo, submit 28-Aug</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
         <is>
           <t>Team Lead</t>
         </is>
       </c>
-      <c r="F34" s="12" t="n">
+      <c r="F34" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G34" s="12" t="n">
+      <c r="G34" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H34" s="12" t="inlineStr">
+      <c r="H34" s="9" t="inlineStr">
         <is>
           <t>T-28</t>
         </is>
@@ -3167,7 +3160,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
@@ -3181,14 +3174,14 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CoachAI — Daily Stand-up Log (Jun–Aug 2026, 6 Sprints)</t>
+          <t>CoachAI - Daily Stand-up Log (Jun-Aug 2026, 6 Sprints)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Daily 15-min stand-ups: Yesterday / Today / Blockers — Scrum Master: Team Lead | Meeting time: 10:00 AM IST | Tool: Google Meet + GitHub Projects</t>
+          <t>Daily 15-min stand-ups: Yesterday / Today / Blockers - Scrum Master: Team Lead | 10:00 AM IST | Google Meet + GitHub Projects</t>
         </is>
       </c>
     </row>
@@ -3250,12 +3243,12 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Kick-off, requirement analysis, created GitHub repo &amp; README skeleton</t>
+          <t>Kick-off, requirement analysis, created GitHub repo and README skeleton</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Finalize architecture diagram &amp; per-turn flow, create .env.example</t>
+          <t>Finalize architecture diagram and per-turn flow, create .env.example</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -3270,37 +3263,37 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Implemented config.py with 3-layer key fallback, tested graceful degradation</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>Start Orchestrator singleton &amp; ConversationManager skeleton</t>
-        </is>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>Azure key not yet provisioned — using Groq fallback</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Implemented config.py with 3-layer key fallback, graceful degradation tested</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Start Orchestrator singleton and ConversationManager skeleton</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>Azure key not yet provisioned - using Groq fallback</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>Request Azure OpenAI access</t>
         </is>
@@ -3324,12 +3317,12 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Completed Orchestrator session lifecycle &amp; DB schema (sessions full_state JSON)</t>
+          <t>Completed Orchestrator lifecycle and DB schema (sessions full_state JSON)</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Wire Streamlit sidebar &amp; setup page</t>
+          <t>Wire Streamlit sidebar and setup page</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -3344,39 +3337,39 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>Built customer_simulator (Hinglish, sentiment machine) + intent_sentiment (JSON regex fallback)</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Built customer_simulator (Hinglish, sentiment) + intent_sentiment (JSON regex fallback)</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Build escalation_monitor weighted formula + unit tests</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
-        <is>
-          <t>LLM occasionally returns markdown fence — added regex extractor</t>
-        </is>
-      </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>Refine prompt for JSON-only output</t>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>LLM returns markdown fence - added regex extractor</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>Refine prompt for JSON-only</t>
         </is>
       </c>
     </row>
@@ -3403,52 +3396,52 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Implement post_interaction_summary scoring formula &amp; report JSON</t>
+          <t>Implement post_interaction_summary scoring and report JSON</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Coaching clarity score variance high — tuning tone heuristics</t>
+          <t>Clarity score variance high - tuning heuristics</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Add heuristic fallback for clarity</t>
+          <t>Add fallback for clarity</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>2026-07-18</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 2 review: 5/5 US completed, demo of &lt;0.5s per-turn pipeline</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 2 review: 5/5 US done, demo &lt;0.5s pipeline</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Begin Sprint 3: RAG ingestion multi-format</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G10" s="13" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>Sprint 3 planning</t>
         </is>
@@ -3472,17 +3465,17 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Ingest implemented (.txt/.pdf via PyPDF2, 512-char chunks), 19 FAQs loaded</t>
+          <t>Ingest .txt/.pdf via PyPDF2, 512-char chunks, 19 FAQs loaded</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Build hybrid retrieval (embedding + BM25) &amp; JSONB cache</t>
+          <t>Build hybrid retrieval (embedding + BM25) and JSONB cache</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>OpenRouter embedding intermittent 429 — keyword fallback saves demo</t>
+          <t>OpenRouter 429 - keyword fallback saved demo</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -3492,39 +3485,39 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Knowledge recommendation + KB-gap &lt;0.45 done, auto-KB draft writes to pending/</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
-          <t>Implement deep_analysis one-call consolidation &amp; 4 risk agents</t>
-        </is>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>Deep analysis prompt too long — split but keep single call</t>
-        </is>
-      </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>Compress prompt, keep structured JSON contract</t>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Knowledge recommendation + KB-gap &lt;0.45 done, auto-KB draft to pending/</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Implement deep_analysis one-call and 4 risk agents</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Deep prompt too long - compress but keep single call</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Compress prompt, keep JSON contract</t>
         </is>
       </c>
     </row>
@@ -3546,12 +3539,12 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Deep signals working, verified predicted CSAT vs heuristic fallback</t>
+          <t>Deep signals working, CSAT vs heuristic verified</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Testing RAG relevance on 30 queries, tuning 0.45 threshold</t>
+          <t>Test RAG on 30 queries, tune 0.45 threshold</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -3566,39 +3559,39 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>Built mind_reader, multiverse, cognitive_load, patience_clock, bot_agent menu logic</t>
-        </is>
-      </c>
-      <c r="E14" s="13" t="inlineStr">
-        <is>
-          <t>Implement manager_supervisor (0.5 threshold), compliance, tone rewriter</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="inlineStr">
-        <is>
-          <t>Manager whisper firing too often — raised threshold 0.5</t>
-        </is>
-      </c>
-      <c r="G14" s="13" t="inlineStr">
-        <is>
-          <t>Adjust to 0.5, add hysteresis</t>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Built mind_reader, multiverse, cognitive_load, patience_clock, bot Agent menu</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Implement manager_supervisor (0.5), compliance, tone rewriter</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>Manager whisper too frequent - raised to 0.5</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>Adjust threshold, add hysteresis</t>
         </is>
       </c>
     </row>
@@ -3620,59 +3613,59 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Tone rewriter &lt;10 char guard done, auto_pilot + Composio mock working</t>
+          <t>Tone rewriter &lt;10 guard done, auto_pilot + Composio mock working</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Build Jira bug generator, scenario generator, QA audit (21 checks)</t>
+          <t>Build Jira generator, scenario generator, QA audit (21 checks)</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Composio SDK version bump broke import — pinned to 0.18.1</t>
+          <t>Composio SDK breaking change 0.18-&gt;0.19</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Pin deps in requirements.txt</t>
+          <t>Pin deps to 0.18.1</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>Backend Team</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
-        <is>
-          <t>Survival Mode arcade &amp; Hall of Fame archiver done, tested power-ups</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 4 review, start Node backend auth &amp; sessionStore</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
-        <is>
-          <t>Survival singleton shared across users — known, document as limitation</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="inlineStr">
-        <is>
-          <t>Add comment in gotchas</t>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Survival arcade and Hall of Fame done, power-ups tested</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 4 review, start Node backend auth and sessionStore</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Survival singleton shared - known limitation</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>Document in gotchas</t>
         </is>
       </c>
     </row>
@@ -3694,17 +3687,17 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Node Express backend: auth (register/login/guest), pg rehydration, 20 routes, health check</t>
+          <t>Node Express backend: auth (register/login/guest), pg rehydration, 20 routes, health</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Build React frontend shell (Landing/Login/Dashboard) &amp; bearer wrapper</t>
+          <t>Build React frontend shell (Landing/Login/Dashboard) and bearer wrapper</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Two backends on same Vercel project — careful deploy order</t>
+          <t>Two backends same Vercel project - deploy order careful</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -3714,37 +3707,37 @@
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Frontend Team</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Frontend Dashboard 4-tab rail (Signals/KB/Reply/Risk) + coaching console wired to /api/chat/message</t>
-        </is>
-      </c>
-      <c r="E18" s="13" t="inlineStr">
-        <is>
-          <t>Implement Feature Lab, Analytics, Reports, Knowledge admin tabs</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>Risk tab overflow on mobile — fixed with Tailwind overflow</t>
-        </is>
-      </c>
-      <c r="G18" s="13" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard 4-tab rail (Signals/KB/Reply/Risk) wired to /api/chat/message</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Implement Feature Lab, Analytics, Reports, Knowledge admin</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Risk tab overflow on mobile - fixed Tailwind</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>Test responsive at 360px</t>
         </is>
@@ -3768,59 +3761,59 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Feature Lab (Multiverse/Tone/Compliance/Jira) + autopilot &amp; manager-takeover flows done</t>
+          <t>Feature Lab (Multiverse/Tone/Compliance/Jira) + autopilot/takeover done</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>End-to-end guest→Setup→Dashboard→Report→Email test</t>
+          <t>End-to-end guest-&gt;Setup-&gt;Dashboard-&gt;Report-&gt;Email test</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>DB rehydration on cold start verified via Neon logs</t>
+          <t>DB rehydration on cold start verified</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Add activity log for audit</t>
+          <t>Add activity log</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>QA Team</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
-        <is>
-          <t>Wrote pytest 14 tests (agents, RAG, load), vitest 7, node --test — all green locally</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>Deploy to Vercel prod &amp; Streamlit Cloud, configure DATABASE_URL</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr">
-        <is>
-          <t>Ephemeral FS caused missing reports — switched to DB authoritative read</t>
-        </is>
-      </c>
-      <c r="G20" s="13" t="inlineStr">
-        <is>
-          <t>Fix: never read from fs on Vercel handlers</t>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>pytest 14 tests + vitest 7 + node --test all green locally</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Deploy to Vercel prod and Streamlit Cloud, configure DATABASE_URL</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Ephemeral FS caused missing reports - switched to DB</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>Never read from fs on Vercel</t>
         </is>
       </c>
     </row>
@@ -3842,7 +3835,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Drafted PPT 10 slides (exactly), KT Guide + Deep Dive, HTML docs</t>
+          <t>Drafted PPT 10 slides exactly, KT Guide + Deep Dive, HTML docs</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -3852,49 +3845,49 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>PPT had 12 slides — trimmed to 10 per Infosys guideline</t>
+          <t>PPT had 12 slides - trimmed to 10</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Enforce 10-slide rule, use Appendix if needed</t>
+          <t>Enforce 10-slide rule</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>QA Team</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>Load test: 50 concurrent chat turns, p95 &lt;0.8s, fallback chain reliable (Azure→Groq)</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="inlineStr">
-        <is>
-          <t>Fill Agile/Defect/UTP templates, final GitHub push to final/main</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
-        <is>
-          <t>.gitignore was ignoring Doc PDFs — fixed with !Doc/**/*.pdf</t>
-        </is>
-      </c>
-      <c r="G22" s="13" t="inlineStr">
-        <is>
-          <t>Verify git status shows PDFs tracked</t>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>Load test 50 concurrent, p95 &lt;0.8s, fallback chain reliable (Azure-&gt;Groq)</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>Fill Agile/Defect/UTP templates, final push to final/main</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>.gitignore ignored Doc PDFs - fixed with !Doc/**/*.pdf</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>Verify git status PDFs tracked</t>
         </is>
       </c>
     </row>
@@ -3916,22 +3909,22 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Completed all templates, final review, presentation dry-run (10min + 5min Q&amp;A)</t>
+          <t>Completed templates, final review, 10min + 5min Q&amp;A dry-run</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Submit to Classroom &amp; GitHub by 28-Aug deadline</t>
+          <t>Submit to Classroom and GitHub by 28-Aug</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>None — submission ready</t>
+          <t>None - submission ready</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Upload &amp; verify GitHub visible</t>
+          <t>Upload and verify</t>
         </is>
       </c>
     </row>
@@ -3954,7 +3947,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
@@ -3967,14 +3960,14 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CoachAI — Sprint Retrospectives (6 Sprints)</t>
+          <t>CoachAI - Sprint Retrospectives (6 Sprints)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>What went well / What went wrong / Improvements — reviewed at each sprint review, owner &amp; due date tracked</t>
+          <t>What went well / What went wrong / Improvements - reviewed at each sprint review</t>
         </is>
       </c>
     </row>
@@ -3989,12 +3982,12 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>What Went Well 😊</t>
+          <t>What Went Well</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>What Went Wrong / Challenges 😞</t>
+          <t>What Went Wrong / Challenges</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -4017,26 +4010,22 @@
       <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Sprint 1
-07–12 Jul 2026</t>
+07-12 Jul 2026</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>• Clear architecture &amp; per-turn flow diagram saved rework
-• Graceful degradation design prevented late surprises
-• GitHub branching clean, README got praise</t>
+          <t>Clear architecture and 9-step flow saved rework; Graceful degradation prevented late surprises; GitHub branching clean</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>• Azure OpenAI access delayed — had to start with Groq
-• Initial chunk size 1024 was too large, truncated tips</t>
+          <t>Azure access delayed - started with Groq; Initial chunk 1024 too large, truncated tips</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>→ Request Azure key early; reduce chunk to 512 &amp; sentence re-split
-→ Document 3-layer key fallback in .env.example</t>
+          <t>Request Azure key early; reduce chunk to 512 and sentence re-split; document 3-layer fallback</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -4047,7 +4036,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>12-Jul • Done</t>
+          <t>12-Jul Done</t>
         </is>
       </c>
     </row>
@@ -4055,37 +4044,33 @@
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Sprint 2
-14–19 Jul 2026</t>
+14-19 Jul 2026</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>• &lt;0.5s per-turn pipeline achieved with ThreadPool 2 workers
-• Escalation weighted formula easy to tune &amp; test
-• Coaching macros library made suggestions product-specific</t>
+          <t>&lt;0.5s pipeline with ThreadPool 2 workers; Escalation formula easy to tune and test; Macros library made suggestions product-specific</t>
         </is>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
-          <t>• LLM JSON parsing failed when model added ```json fences
-• Clarity score variance across intents</t>
+          <t>LLM JSON failed when model added ```json fences; Clarity score variance across intents</t>
         </is>
       </c>
       <c r="D6" s="17" t="inlineStr">
         <is>
-          <t>→ Add regex JSON extractor + heuristic fallback for every LLM agent
-→ Tune coaching prompt to inject valid intents enum + calibrate thresholds</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
+          <t>Add regex JSON extractor + heuristic fallback for every agent; Tune coaching prompt with valid intents enum</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>AI Team
 QA Team</t>
         </is>
       </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>19-Jul • Done</t>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>19-Jul Done</t>
         </is>
       </c>
     </row>
@@ -4093,26 +4078,22 @@
       <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Sprint 3
-21–26 Jul 2026</t>
+21-26 Jul 2026</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>• Hybrid RAG (semantic+BM25) works offline — demo never dead
-• KB-gap &lt;0.45 detection + auto-KB draft delighted reviewers
-• Deep analysis one-call consolidation cut latency 40%</t>
+          <t>Hybrid RAG (semantic+BM25) works offline; KB-gap &lt;0.45 + auto-KB draft delighted reviewers; Deep one-call cut latency 40%</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>• OpenRouter 429 rate-limit spiked during demo
-• Viral/fraud keyword pre-scan false negatives on Hinglish</t>
+          <t>OpenRouter 429 during demo; Viral/fraud keyword false negatives on Hinglish</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>→ Add retry + keyword fallback seeded defaults + log so UI degrades not breaks
-→ Expand Hinglish keyword lists, add tests for “paise wapas” etc.</t>
+          <t>Add retry + keyword seeded defaults + log; Expand Hinglish lists, tests for 'paise wapas'</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -4122,7 +4103,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>26-Jul • Done</t>
+          <t>26-Jul Done</t>
         </is>
       </c>
     </row>
@@ -4130,39 +4111,33 @@
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Sprint 4
-28 Jul–02 Aug</t>
+28 Jul-02 Aug</t>
         </is>
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>• 25 agents all with single responsibility — prompts small &amp; testable
-• Composio Jira/Gmail/Slack real actions impressed; mock keeps demo offline
-• Survival Mode &amp; Hall of Fame added gamified training wow factor</t>
+          <t>25 agents single responsibility - prompts small/testable; Composio real actions + mock offline; Survival and Hall of Fame wow factor</t>
         </is>
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
-          <t>• Composio SDK breaking change (0.18→0.19) broke imports
-• Manager whisper fired on every frustrated message — noisy
-• Survival singleton shared across users</t>
+          <t>Composio SDK breaking change 0.18-&gt;0.19; Manager whisper fired too often (&gt;0.3); Survival singleton shared</t>
         </is>
       </c>
       <c r="D8" s="17" t="inlineStr">
         <is>
-          <t>→ Pin composio&gt;=0.18.1,&lt;0.20 in requirements.txt
-→ Add fast-path no-op unless ≥0.5 + hysteresys; document singleton limit in gotchas
-→ QA audit 21 checks stabilized scoring</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
+          <t>Pin composio&gt;=0.18.1,&lt;0.20; Raise threshold to &gt;=0.5 + hysteresis; Document singleton limit in gotchas</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>AI Team
 Backend Team</t>
         </is>
       </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>02-Aug • Done</t>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>02-Aug Done</t>
         </is>
       </c>
     </row>
@@ -4170,28 +4145,22 @@
       <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Sprint 5
-04–09 Aug 2026</t>
+04-09 Aug 2026</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>• Node backend mirrors Python agents — frontend auth finally works (/api/auth/*)
-• React 4-tab rail (Signals/KB/Reply/Risk) rated highly usable
-• Feature Lab multiverse &amp; tone rewriter are strong demo moments</t>
+          <t>Node backend mirrors Python - frontend auth works (/api/auth/*); React 4-tab rail highly usable; Feature Lab strong demo</t>
         </is>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>• Two backends on same Vercel project caused deploy confusion
-• Risk tab overflow on mobile, auth token expiry not redirecting
-• DB rehydration edge: cold instance lost in-memory _sessions</t>
+          <t>Two backends same Vercel project confusion; Risk tab overflow mobile; DB rehydration edge: cold instance lost _sessions</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>→ Deploy Node to coachai-backend, verify /health before frontend deploy
-→ Fix responsive Tailwind overflow, add auth redirect + JSON rehydrate via full_state
-→ Add activity log &amp; persist session on every turn</t>
+          <t>Deploy Node to coachai-backend, verify /health before frontend; Fix responsive; Add JSON rehydrate via full_state + activity log</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -4202,7 +4171,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>09-Aug • Done</t>
+          <t>09-Aug Done</t>
         </is>
       </c>
     </row>
@@ -4210,47 +4179,41 @@
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Sprint 6
-11–27 Aug 2026</t>
+11-27 Aug 2026</t>
         </is>
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>• Full test suite green (pytest+vitest+node), p95 &lt;0.8s under load
-• 10-slide PPT exactly + KT Guide + QA Bank ready for viva
-• Ephemeral FS fix (DB authoritative) closed top production bug</t>
+          <t>Full suite green (pytest+vitest+node), p95 &lt;0.8s; 10-slide PPT exactly + KT Guide + QA Bank ready; Ephemeral FS fix closed top bug</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t>• PPT initially 12 slides — had to trim (Infosys requires exactly 10)
-• .gitignore ignored Doc PDFs — almost missed submission assets
-• Last-minute template filling for Agile/Defect/UTP took a full day</t>
+          <t>PPT initially 12 slides - had to trim; .gitignore ignored Doc PDFs - almost missed; Template filling took full day</t>
         </is>
       </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
-          <t>→ Enforce slide count in review checklist; add !Doc/**/*.pdf to .gitignore
-→ Create template-filling script (this workbook generator) for next batch
-→ Final dry-run 27-Aug, submit 28-Aug before 11:59 PM</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
+          <t>Enforce slide count checklist; Add !Doc/**/*.pdf; Create generator script for next batch; Dry-run 27-Aug, submit 28-Aug</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>Team Lead
 QA Team
 All</t>
         </is>
       </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>27-Aug • Done</t>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>27-Aug Done</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Retrospective outcome: 30/30 user stories completed, 0 blockers pending, velocity stable (~5 stories/sprint). Key lesson: two-backends-one-Vercel-project &amp; ephemeral FS were the top architectural risks — mitigated via pg JSONB rehydration &amp; DB-authoritative reads. Next: unify to single canonical backend, add pgvector at scale.</t>
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Outcome: 30/30 user stories completed, 0 blockers pending, velocity ~5 stories/sprint. Top risks mitigated: two-backends-one-Vercel and ephemeral FS via pg JSONB rehydration and DB-authoritative reads. Next: unify to single canonical backend, add pgvector at scale.</t>
         </is>
       </c>
     </row>

</xml_diff>